<commit_message>
mapa: perguntas enxutas (máx. 13 palavras) + quiz estilo Typeform
- 36 perguntas reescritas na versão enxuta no xlsx (fonte de verdade) e
  catálogo regenerado; voz afirmativa e sujeito preservados
- MM2-MAR-10b agora limita a 3 atributos (texto "escolha até 3" + trava na UI)
- /mapa/[token]: uma afirmação por tela, auto-avanço 320ms ao tocar na
  resposta, botão voltar; "Continuar" só na múltipla escolha
- checkpoint de respostas por bloco + save completo antes do finalize

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/diagnostic-web/data/maturidade/mapa_maturidade_final.xlsx
+++ b/apps/diagnostic-web/data/maturidade/mapa_maturidade_final.xlsx
@@ -936,7 +936,7 @@
       </c>
       <c r="G2" s="17" t="inlineStr">
         <is>
-          <t>Clientes e potenciais clientes chegam até a empresa já entendendo minimamente o que ela faz.</t>
+          <t>Clientes chegam até a empresa já entendendo o que ela faz.</t>
         </is>
       </c>
       <c r="H2" s="17" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>As pessoas confiam na empresa desde os primeiros contatos, mesmo antes de comprar.</t>
+          <t>As pessoas confiam na empresa desde os primeiros contatos.</t>
         </is>
       </c>
       <c r="H4" s="17" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>A empresa recebe indicações espontâneas de clientes, parceiros ou pessoas do mercado.</t>
+          <t>A empresa recebe indicações espontâneas de clientes, parceiros ou mercado.</t>
         </is>
       </c>
       <c r="H5" s="17" t="inlineStr">
@@ -1268,7 +1268,7 @@
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>Clientes que já compraram tendem a considerar a empresa novamente em uma necessidade semelhante.</t>
+          <t>Quem já comprou volta a considerar a empresa em necessidades semelhantes.</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>A forma como a empresa se apresenta é consistente nos canais, materiais e propostas comerciais.</t>
+          <t>A apresentação da empresa é consistente em canais, materiais e propostas.</t>
         </is>
       </c>
       <c r="H7" s="17" t="inlineStr">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>A empresa apresenta evidências claras de sua capacidade, como resultados, cases, depoimentos ou histórico.</t>
+          <t>A empresa mostra evidências claras de capacidade: resultados, cases, depoimentos.</t>
         </is>
       </c>
       <c r="H8" s="17" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>A reputação da empresa facilita a abertura de conversas e novas oportunidades.</t>
+          <t>A reputação da empresa abre conversas e novas oportunidades.</t>
         </is>
       </c>
       <c r="H9" s="17" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>A empresa desperta interesse em bons profissionais, parceiros ou fornecedores estratégicos.</t>
+          <t>A empresa desperta interesse em bons profissionais, parceiros e fornecedores.</t>
         </is>
       </c>
       <c r="H10" s="17" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>Quando falam da empresa, as pessoas a associam a adjetivos positivos.</t>
+          <t>Quando falam da empresa, as pessoas usam adjetivos positivos.</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>A quais adjetivos as pessoas mais associam a empresa hoje? (marque os que se aplicam)</t>
+          <t>Quais adjetivos as pessoas mais associam à empresa hoje? (escolha até 3)</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>As principais decisões da rotina estão conectadas às prioridades do negócio.</t>
+          <t>As decisões da rotina estão conectadas às prioridades do negócio.</t>
         </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>A empresa possui uma rotina consistente para gerar novas oportunidades comerciais.</t>
+          <t>A empresa tem rotina consistente para gerar novas oportunidades comerciais.</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>A empresa consegue recusar demandas, projetos ou clientes que desviam o foco do que é prioritário.</t>
+          <t>A empresa consegue recusar demandas que desviam o foco do prioritário.</t>
         </is>
       </c>
       <c r="H15" s="17" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>A empresa acompanha se cada venda, contrato ou projeto gera margem adequada.</t>
+          <t>A empresa acompanha se cada venda ou projeto gera margem adequada.</t>
         </is>
       </c>
       <c r="H16" s="17" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>A empresa cumpre prazos, condições e entregas combinadas com os clientes.</t>
+          <t>A empresa cumpre prazos, condições e entregas combinadas.</t>
         </is>
       </c>
       <c r="H17" s="17" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="G18" s="17" t="inlineStr">
         <is>
-          <t>As rotinas críticas do negócio possuem padrão mínimo de execução.</t>
+          <t>As rotinas críticas do negócio têm padrão mínimo de execução.</t>
         </is>
       </c>
       <c r="H18" s="17" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
-          <t>A empresa acompanha indicadores essenciais de vendas, margem, caixa, produtividade e satisfação.</t>
+          <t>A empresa acompanha indicadores de vendas, margem, caixa e satisfação.</t>
         </is>
       </c>
       <c r="H19" s="17" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="G20" s="17" t="inlineStr">
         <is>
-          <t>A empresa consegue atender a demanda atual sem sobrecarga excessiva ou perda de qualidade.</t>
+          <t>A empresa atende a demanda atual sem sobrecarga nem perda de qualidade.</t>
         </is>
       </c>
       <c r="H20" s="17" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>As reuniões e acompanhamentos terminam com decisões, responsáveis e próximos passos claros.</t>
+          <t>Reuniões terminam com decisões, responsáveis e próximos passos claros.</t>
         </is>
       </c>
       <c r="H21" s="17" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="G22" s="17" t="inlineStr">
         <is>
-          <t>A empresa consegue crescer sem aumentar excessivamente a dependência dos sócios.</t>
+          <t>A empresa cresce sem aumentar a dependência dos sócios.</t>
         </is>
       </c>
       <c r="H22" s="17" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
-          <t>As pessoas entendem com clareza quais são as prioridades da empresa no momento.</t>
+          <t>As pessoas entendem com clareza as prioridades atuais da empresa.</t>
         </is>
       </c>
       <c r="H23" s="17" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>Os repasses entre áreas são claros o suficiente para evitar retrabalho e falhas na entrega.</t>
+          <t>Os repasses entre áreas evitam retrabalho e falhas na entrega.</t>
         </is>
       </c>
       <c r="H25" s="17" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>As propostas comerciais deixam claro escopo, valor, prazo, condições e próximos passos.</t>
+          <t>As propostas deixam claros escopo, valor, prazo e próximos passos.</t>
         </is>
       </c>
       <c r="H26" s="17" t="inlineStr">
@@ -3007,7 +3007,7 @@
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
-          <t>É fácil para um cliente entender os produtos, serviços ou soluções oferecidos pela empresa.</t>
+          <t>É fácil para o cliente entender o que a empresa oferece.</t>
         </is>
       </c>
       <c r="H27" s="17" t="inlineStr">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>Durante a entrega, o cliente recebe informações suficientes sobre andamento, prazos e próximos passos.</t>
+          <t>Durante a entrega, o cliente sabe andamento, prazos e próximos passos.</t>
         </is>
       </c>
       <c r="H28" s="17" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
-          <t>Quando surgem mudanças, atrasos ou problemas, a empresa comunica com transparência e agilidade.</t>
+          <t>Mudanças, atrasos ou problemas são comunicados com transparência e agilidade.</t>
         </is>
       </c>
       <c r="H29" s="17" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="G30" s="17" t="inlineStr">
         <is>
-          <t>A empresa possui canais claros para comunicar decisões, demandas, mudanças e informações importantes.</t>
+          <t>A empresa tem canais claros para comunicar decisões e mudanças.</t>
         </is>
       </c>
       <c r="H30" s="17" t="inlineStr">
@@ -3422,7 +3422,7 @@
       </c>
       <c r="G32" s="17" t="inlineStr">
         <is>
-          <t>A empresa transforma os feedbacks dos clientes em melhorias concretas — não fica só na escuta.</t>
+          <t>A empresa transforma feedbacks de clientes em melhorias concretas.</t>
         </is>
       </c>
       <c r="H32" s="17" t="inlineStr">
@@ -3588,7 +3588,7 @@
       </c>
       <c r="G34" s="17" t="inlineStr">
         <is>
-          <t>As pessoas conseguem tomar decisões compatíveis com suas responsabilidades.</t>
+          <t>As pessoas tomam decisões compatíveis com suas responsabilidades.</t>
         </is>
       </c>
       <c r="H34" s="17" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>As lideranças acompanham entregas, prioridades e obstáculos da equipe com frequência.</t>
+          <t>As lideranças acompanham entregas, prioridades e obstáculos com frequência.</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
@@ -3754,7 +3754,7 @@
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t>A equipe consegue entregar o que é prioritário sem viver em constante urgência.</t>
+          <t>A equipe entrega o prioritário sem viver em constante urgência.</t>
         </is>
       </c>
       <c r="H36" s="17" t="inlineStr">
@@ -3837,7 +3837,7 @@
       </c>
       <c r="G37" s="17" t="inlineStr">
         <is>
-          <t>As pessoas demonstram preparo técnico e comportamental para realizar bem suas funções.</t>
+          <t>As pessoas têm preparo técnico e comportamental para suas funções.</t>
         </is>
       </c>
       <c r="H37" s="17" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="G38" s="17" t="inlineStr">
         <is>
-          <t>O cliente recebe um padrão de atendimento consistente, independentemente da pessoa ou canal.</t>
+          <t>O atendimento ao cliente é consistente, independentemente da pessoa ou canal.</t>
         </is>
       </c>
       <c r="H38" s="17" t="inlineStr">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="G39" s="17" t="inlineStr">
         <is>
-          <t>A direção delega decisões e as respeita, sem retomar o controle a todo momento.</t>
+          <t>A direção delega decisões e as respeita, sem retomar o controle.</t>
         </is>
       </c>
       <c r="H39" s="17" t="inlineStr">
@@ -4169,7 +4169,7 @@
       </c>
       <c r="G41" s="17" t="inlineStr">
         <is>
-          <t>A empresa consegue manter profissionais importantes para a operação e o crescimento.</t>
+          <t>A empresa retém os profissionais importantes para operação e crescimento.</t>
         </is>
       </c>
       <c r="H41" s="17" t="inlineStr">
@@ -4252,7 +4252,7 @@
       </c>
       <c r="G42" s="17" t="inlineStr">
         <is>
-          <t>Os líderes dedicam tempo a pensar o futuro do negócio, e não apenas a resolver o operacional do dia a dia.</t>
+          <t>Os líderes dedicam tempo a pensar o futuro do negócio.</t>
         </is>
       </c>
       <c r="H42" s="17" t="inlineStr">

</xml_diff>